<commit_message>
vMay24 - CMS + DNA fingerprinting
</commit_message>
<xml_diff>
--- a/Output/Tables/tab_oaxaca_FM.xlsx
+++ b/Output/Tables/tab_oaxaca_FM.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="98">
-  <si>
-    <t>ICV_Managed_self</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="95">
+  <si>
+    <t>selfMagIcv</t>
   </si>
   <si>
     <t>Wives</t>
@@ -40,31 +40,25 @@
     <t>constant</t>
   </si>
   <si>
-    <t>Coop_self</t>
+    <t>Coop Member</t>
   </si>
   <si>
     <t>Household Credit</t>
   </si>
   <si>
-    <t>Extension_Access_self</t>
-  </si>
-  <si>
-    <t>Cell_Own_self</t>
-  </si>
-  <si>
-    <t>Fertilizer</t>
-  </si>
-  <si>
-    <t>Consumption (%)</t>
-  </si>
-  <si>
-    <t>Zone 1</t>
-  </si>
-  <si>
-    <t>Zone 3</t>
-  </si>
-  <si>
-    <t>Zone 4</t>
+    <t>Extension Access</t>
+  </si>
+  <si>
+    <t>Consump perc</t>
+  </si>
+  <si>
+    <t>Zone1</t>
+  </si>
+  <si>
+    <t>Zone3</t>
+  </si>
+  <si>
+    <t>Zone4</t>
   </si>
   <si>
     <t>Age</t>
@@ -82,232 +76,229 @@
     <t>(Base)</t>
   </si>
   <si>
-    <t>0.167</t>
-  </si>
-  <si>
-    <t>0.647</t>
-  </si>
-  <si>
-    <t>-0.480</t>
+    <t>0.086</t>
+  </si>
+  <si>
+    <t>0.324</t>
+  </si>
+  <si>
+    <t>-0.238</t>
   </si>
   <si>
     <t>endowments</t>
   </si>
   <si>
-    <t>-0.053</t>
+    <t>-0.051</t>
+  </si>
+  <si>
+    <t>(0.064)</t>
+  </si>
+  <si>
+    <t>5.69\%</t>
+  </si>
+  <si>
+    <t>-0.000</t>
+  </si>
+  <si>
+    <t>(0.000)</t>
+  </si>
+  <si>
+    <t>0.007</t>
+  </si>
+  <si>
+    <t>(0.007)</t>
+  </si>
+  <si>
+    <t>0.009</t>
+  </si>
+  <si>
+    <t>(0.010)</t>
+  </si>
+  <si>
+    <t>-0.062 ***</t>
+  </si>
+  <si>
+    <t>(0.020)</t>
+  </si>
+  <si>
+    <t>0.006</t>
+  </si>
+  <si>
+    <t>(0.004)</t>
+  </si>
+  <si>
+    <t>0.001</t>
+  </si>
+  <si>
+    <t>-0.002</t>
+  </si>
+  <si>
+    <t>0.020</t>
+  </si>
+  <si>
+    <t>(0.048)</t>
+  </si>
+  <si>
+    <t>-0.017</t>
+  </si>
+  <si>
+    <t>(0.016)</t>
+  </si>
+  <si>
+    <t>-0.013</t>
+  </si>
+  <si>
+    <t>(0.009)</t>
+  </si>
+  <si>
+    <t>0.002</t>
+  </si>
+  <si>
+    <t>(0.006)</t>
+  </si>
+  <si>
+    <t>-0.001</t>
+  </si>
+  <si>
+    <t>(0.017)</t>
+  </si>
+  <si>
+    <t>coefficients</t>
+  </si>
+  <si>
+    <t>-0.723 ***</t>
+  </si>
+  <si>
+    <t>(0.126)</t>
+  </si>
+  <si>
+    <t>80.69\%</t>
+  </si>
+  <si>
+    <t>-1.235 ***</t>
+  </si>
+  <si>
+    <t>(0.472)</t>
+  </si>
+  <si>
+    <t>-0.136 **</t>
+  </si>
+  <si>
+    <t>(0.055)</t>
+  </si>
+  <si>
+    <t>0.051</t>
+  </si>
+  <si>
+    <t>(0.089)</t>
+  </si>
+  <si>
+    <t>-0.188 **</t>
+  </si>
+  <si>
+    <t>(0.088)</t>
+  </si>
+  <si>
+    <t>0.096</t>
+  </si>
+  <si>
+    <t>(0.205)</t>
+  </si>
+  <si>
+    <t>-0.056</t>
+  </si>
+  <si>
+    <t>(0.044)</t>
+  </si>
+  <si>
+    <t>0.104 ***</t>
+  </si>
+  <si>
+    <t>(0.036)</t>
+  </si>
+  <si>
+    <t>0.746 *</t>
+  </si>
+  <si>
+    <t>(0.432)</t>
+  </si>
+  <si>
+    <t>0.071</t>
+  </si>
+  <si>
+    <t>(0.187)</t>
+  </si>
+  <si>
+    <t>-0.037</t>
+  </si>
+  <si>
+    <t>(0.210)</t>
+  </si>
+  <si>
+    <t>-0.023</t>
+  </si>
+  <si>
+    <t>-0.123 **</t>
   </si>
   <si>
     <t>(0.052)</t>
   </si>
   <si>
-    <t>11.04\%</t>
+    <t>interaction</t>
+  </si>
+  <si>
+    <t>-0.122</t>
+  </si>
+  <si>
+    <t>(0.101)</t>
+  </si>
+  <si>
+    <t>13.62\%</t>
+  </si>
+  <si>
+    <t>-0.018</t>
+  </si>
+  <si>
+    <t>-0.008</t>
+  </si>
+  <si>
+    <t>(0.015)</t>
+  </si>
+  <si>
+    <t>0.068 **</t>
+  </si>
+  <si>
+    <t>(0.033)</t>
+  </si>
+  <si>
+    <t>-0.003</t>
+  </si>
+  <si>
+    <t>(0.008)</t>
   </si>
   <si>
     <t>0.000</t>
   </si>
   <si>
-    <t>(0.000)</t>
-  </si>
-  <si>
-    <t>-0.009</t>
-  </si>
-  <si>
-    <t>(0.008)</t>
-  </si>
-  <si>
-    <t>0.002</t>
-  </si>
-  <si>
-    <t>(0.007)</t>
-  </si>
-  <si>
-    <t>-0.044 *</t>
-  </si>
-  <si>
-    <t>(0.026)</t>
-  </si>
-  <si>
-    <t>0.017 *</t>
-  </si>
-  <si>
-    <t>(0.010)</t>
-  </si>
-  <si>
-    <t>(0.002)</t>
-  </si>
-  <si>
-    <t>0.004</t>
-  </si>
-  <si>
     <t>(0.005)</t>
   </si>
   <si>
-    <t>-0.000</t>
-  </si>
-  <si>
-    <t>(0.004)</t>
-  </si>
-  <si>
-    <t>0.006</t>
-  </si>
-  <si>
-    <t>(0.032)</t>
-  </si>
-  <si>
-    <t>-0.014</t>
-  </si>
-  <si>
-    <t>(0.015)</t>
-  </si>
-  <si>
-    <t>-0.016 *</t>
-  </si>
-  <si>
-    <t>(0.009)</t>
-  </si>
-  <si>
-    <t>-0.001</t>
-  </si>
-  <si>
-    <t>(0.011)</t>
-  </si>
-  <si>
-    <t>coefficients</t>
-  </si>
-  <si>
-    <t>-0.462 ***</t>
-  </si>
-  <si>
-    <t>(0.057)</t>
-  </si>
-  <si>
-    <t>96.25\%</t>
-  </si>
-  <si>
-    <t>-0.532 **</t>
-  </si>
-  <si>
-    <t>(0.241)</t>
-  </si>
-  <si>
-    <t>-0.030 **</t>
-  </si>
-  <si>
-    <t>(0.013)</t>
-  </si>
-  <si>
-    <t>-0.002</t>
-  </si>
-  <si>
-    <t>(0.047)</t>
-  </si>
-  <si>
-    <t>-0.091 ***</t>
-  </si>
-  <si>
-    <t>0.161 ***</t>
-  </si>
-  <si>
-    <t>(0.055)</t>
-  </si>
-  <si>
-    <t>0.029</t>
-  </si>
-  <si>
-    <t>(0.034)</t>
-  </si>
-  <si>
-    <t>0.149</t>
-  </si>
-  <si>
-    <t>(0.102)</t>
-  </si>
-  <si>
-    <t>0.013</t>
-  </si>
-  <si>
-    <t>(0.020)</t>
-  </si>
-  <si>
-    <t>0.018</t>
-  </si>
-  <si>
-    <t>(0.024)</t>
-  </si>
-  <si>
-    <t>0.036 *</t>
-  </si>
-  <si>
-    <t>(0.019)</t>
-  </si>
-  <si>
-    <t>0.287</t>
-  </si>
-  <si>
-    <t>(0.230)</t>
-  </si>
-  <si>
-    <t>-0.062</t>
-  </si>
-  <si>
-    <t>(0.121)</t>
-  </si>
-  <si>
-    <t>-0.335 **</t>
-  </si>
-  <si>
-    <t>(0.133)</t>
-  </si>
-  <si>
-    <t>0.001</t>
+    <t>0.003</t>
   </si>
   <si>
     <t>(0.012)</t>
   </si>
   <si>
-    <t>-0.103 ***</t>
-  </si>
-  <si>
-    <t>(0.031)</t>
-  </si>
-  <si>
-    <t>interaction</t>
-  </si>
-  <si>
-    <t>0.035</t>
-  </si>
-  <si>
-    <t>-7.29\%</t>
-  </si>
-  <si>
-    <t>0.087 ***</t>
-  </si>
-  <si>
-    <t>-0.037 ***</t>
-  </si>
-  <si>
-    <t>(0.003)</t>
-  </si>
-  <si>
-    <t>-0.004</t>
-  </si>
-  <si>
-    <t>(0.006)</t>
-  </si>
-  <si>
-    <t>-0.057</t>
-  </si>
-  <si>
-    <t>(0.046)</t>
-  </si>
-  <si>
-    <t>0.009</t>
-  </si>
-  <si>
-    <t>(0.017)</t>
-  </si>
-  <si>
-    <t>0.020 *</t>
+    <t>-0.150 *</t>
+  </si>
+  <si>
+    <t>-0.010</t>
+  </si>
+  <si>
+    <t>(0.025)</t>
+  </si>
+  <si>
+    <t>(0.014)</t>
   </si>
 </sst>
 </file>
@@ -665,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -684,7 +675,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -692,7 +683,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -700,19 +691,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1"/>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -720,25 +711,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -746,13 +737,13 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -765,25 +756,25 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1"/>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -791,25 +782,25 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1"/>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -817,25 +808,25 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1"/>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -843,22 +834,22 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1"/>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
         <v>84</v>
@@ -869,25 +860,25 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1"/>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -895,25 +886,25 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1"/>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -921,25 +912,25 @@
         <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="D22" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1"/>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="D23" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -947,25 +938,25 @@
         <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1"/>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -973,25 +964,25 @@
         <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>29</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1"/>
       <c r="B27" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D27" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -999,25 +990,25 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1"/>
       <c r="B29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D29" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1025,22 +1016,22 @@
         <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D30" t="s">
-        <v>93</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1"/>
       <c r="B31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C31" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D31" t="s">
         <v>94</v>
@@ -1051,25 +1042,25 @@
         <v>18</v>
       </c>
       <c r="B32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1"/>
       <c r="B33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C33" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1077,77 +1068,25 @@
         <v>19</v>
       </c>
       <c r="B34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C34" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1"/>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D35" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36" t="s">
-        <v>81</v>
-      </c>
-      <c r="D36" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="1"/>
-      <c r="B37" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" t="s">
-        <v>82</v>
-      </c>
-      <c r="D37" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B38" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" t="s">
-        <v>83</v>
-      </c>
-      <c r="D38" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="1"/>
-      <c r="B39" t="s">
-        <v>51</v>
-      </c>
-      <c r="C39" t="s">
-        <v>84</v>
-      </c>
-      <c r="D39" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>